<commit_message>
Redesign constraints API: dict[str, type] for dynamic refs (closes #135) (#147)
* dynamic refs example

* DynamicRef examples

* fix: avoid false-positive dynamic ref errors for static OFFSET and INDIRECT

Classify static OFFSET/INDIRECT calls in default graph extraction so scalar-only expressions resolve without requiring dynamic constraints, and add warning coverage for indeterministic function chains while excluding CELL from that warning path.

Co-authored-by: Cursor <cursoragent@cursor.com>

* Regenerate non-dynamic OFFSET example without cached ref flag

* Redesign constraints API to use plain dict instead of TypedDict

---------

Co-authored-by: chriscarrollsmith <christopher.smith@promptlytechnologies.com>
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/examples/micro-workbook/example-cases.xlsx
+++ b/examples/micro-workbook/example-cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Software\excel-grapher\examples\micro-workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5472DBDE-E73D-4969-BC06-8237B61EDDDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9566D7C9-D1E7-47B0-A06E-B486EA112600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12015" yWindow="0" windowWidth="11985" windowHeight="12780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Formula with no dependencies</t>
   </si>
@@ -57,6 +57,12 @@
   </si>
   <si>
     <t>May cycle</t>
+  </si>
+  <si>
+    <t>OFFSET with scalar arguments</t>
+  </si>
+  <si>
+    <t>OFFSET with dynamic arguments</t>
   </si>
 </sst>
 </file>
@@ -398,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -519,6 +525,39 @@
         <v>1</v>
       </c>
     </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <f ca="1">OFFSET(B9,0,1)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <f ca="1">OFFSET(C10,0,B10)</f>
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Support passing ranges and named ranges as targets to create_dependency_graph
</commit_message>
<xml_diff>
--- a/examples/micro-workbook/example-cases.xlsx
+++ b/examples/micro-workbook/example-cases.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Software\excel-grapher\examples\micro-workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9566D7C9-D1E7-47B0-A06E-B486EA112600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49FE9116-6EAE-465B-8747-5300A12C1587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12015" yWindow="0" windowWidth="11985" windowHeight="12780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="MyNamedRange">Sheet1!$C$11:$D$11</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Formula with no dependencies</t>
   </si>
@@ -63,6 +66,9 @@
   </si>
   <si>
     <t>OFFSET with dynamic arguments</t>
+  </si>
+  <si>
+    <t>Multiple targets</t>
   </si>
 </sst>
 </file>
@@ -404,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -558,6 +564,22 @@
         <v>1</v>
       </c>
     </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <f>B11+1</f>
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <f>B11+2</f>
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Support passing ranges and named ranges as targets to create_dependency_graph (#150)
Co-authored-by: chriscarrollsmith <christopher.smith@promptlytechnologies.com>
</commit_message>
<xml_diff>
--- a/examples/micro-workbook/example-cases.xlsx
+++ b/examples/micro-workbook/example-cases.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Software\excel-grapher\examples\micro-workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9566D7C9-D1E7-47B0-A06E-B486EA112600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49FE9116-6EAE-465B-8747-5300A12C1587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12015" yWindow="0" windowWidth="11985" windowHeight="12780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="MyNamedRange">Sheet1!$C$11:$D$11</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Formula with no dependencies</t>
   </si>
@@ -63,6 +66,9 @@
   </si>
   <si>
     <t>OFFSET with dynamic arguments</t>
+  </si>
+  <si>
+    <t>Multiple targets</t>
   </si>
 </sst>
 </file>
@@ -404,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -558,6 +564,22 @@
         <v>1</v>
       </c>
     </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <f>B11+1</f>
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <f>B11+2</f>
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>